<commit_message>
Actualización de montos de contrapartida y scripts de verificación
</commit_message>
<xml_diff>
--- a/avance0403.xlsx
+++ b/avance0403.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LUCHO\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B5F919-646C-4AAC-8469-88BDC6E91A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BE9D8C-F147-4FCB-8F74-C85B13D1C5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BD18AC21-6960-4AE2-8339-20D741B3F2ED}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$C$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$C$58</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -328,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -355,6 +355,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -691,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D23ADC3-8B94-4C89-9402-4892B6A0FB19}">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="2" customWidth="1"/>
@@ -740,7 +746,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="4">
-        <v>374082</v>
+        <v>416265.13</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -794,8 +800,8 @@
       <c r="B9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="5">
-        <v>91662.8</v>
+      <c r="C9" s="10">
+        <v>137494.20000000001</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -806,7 +812,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="4">
-        <v>78823.98000000001</v>
+        <v>136858.06</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -817,7 +823,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="4">
-        <v>85101.15</v>
+        <v>140456.29999999999</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -839,7 +845,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="4">
-        <v>368965.26</v>
+        <v>468465.26</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -872,7 +878,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="4">
-        <v>96607</v>
+        <v>193214</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1026,7 +1032,7 @@
         <v>28</v>
       </c>
       <c r="C30" s="4">
-        <v>48033.93</v>
+        <v>136330.22</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1037,7 +1043,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="4">
-        <v>395393.22</v>
+        <v>474751.22</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1048,7 +1054,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="4">
-        <v>395030</v>
+        <v>474036</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1092,7 +1098,7 @@
         <v>34</v>
       </c>
       <c r="C36" s="4">
-        <v>143600.17000000001</v>
+        <v>180309.16</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1169,7 +1175,7 @@
         <v>41</v>
       </c>
       <c r="C43" s="8">
-        <v>197046</v>
+        <v>336614</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1326,7 +1332,13 @@
         <v>154810.5</v>
       </c>
     </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C58" s="11"/>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C57">
+    <sortCondition ref="A2:A57"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>